<commit_message>
Data Cleaning: Completamento automatico colonne Comune e Provincia in Excel
</commit_message>
<xml_diff>
--- a/app/src/main/assets/Pipistrelli 2025.xlsx
+++ b/app/src/main/assets/Pipistrelli 2025.xlsx
@@ -527,10 +527,10 @@
         </is>
       </c>
       <c r="H2" t="n">
-        <v>45.50000357045202</v>
+        <v>45.59746520960268</v>
       </c>
       <c r="I2" t="n">
-        <v>11.51809260947295</v>
+        <v>11.54687495840081</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -587,10 +587,10 @@
         </is>
       </c>
       <c r="H3" t="n">
-        <v>45.51660795095754</v>
+        <v>45.50665671632508</v>
       </c>
       <c r="I3" t="n">
-        <v>11.56607306055841</v>
+        <v>11.59015463679549</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -643,10 +643,10 @@
         </is>
       </c>
       <c r="H4" t="n">
-        <v>45.52979483510778</v>
+        <v>45.53089578038835</v>
       </c>
       <c r="I4" t="n">
-        <v>11.52360844193016</v>
+        <v>11.50945956132898</v>
       </c>
       <c r="J4" t="inlineStr">
         <is>
@@ -699,10 +699,10 @@
         </is>
       </c>
       <c r="H5" t="n">
-        <v>45.5285989135124</v>
+        <v>45.54048701756293</v>
       </c>
       <c r="I5" t="n">
-        <v>11.52794494045143</v>
+        <v>11.57704819816247</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -755,10 +755,10 @@
         </is>
       </c>
       <c r="H6" t="n">
-        <v>45.55381514934189</v>
+        <v>45.56546313417498</v>
       </c>
       <c r="I6" t="n">
-        <v>11.49680638576682</v>
+        <v>11.54539076489067</v>
       </c>
       <c r="J6" t="inlineStr">
         <is>
@@ -815,10 +815,10 @@
         </is>
       </c>
       <c r="H7" t="n">
-        <v>45.56240559822008</v>
+        <v>45.5188596165759</v>
       </c>
       <c r="I7" t="n">
-        <v>11.53900136930778</v>
+        <v>11.57135076220658</v>
       </c>
       <c r="J7" t="inlineStr">
         <is>
@@ -871,10 +871,10 @@
         </is>
       </c>
       <c r="H8" t="n">
-        <v>45.51049667069403</v>
+        <v>45.58150146270299</v>
       </c>
       <c r="I8" t="n">
-        <v>11.52418476472131</v>
+        <v>11.54978839303273</v>
       </c>
       <c r="J8" t="inlineStr">
         <is>
@@ -931,10 +931,10 @@
         </is>
       </c>
       <c r="H9" t="n">
-        <v>45.51428556619175</v>
+        <v>45.55409738399385</v>
       </c>
       <c r="I9" t="n">
-        <v>11.51663293698729</v>
+        <v>11.5057750812334</v>
       </c>
       <c r="J9" t="inlineStr">
         <is>
@@ -987,10 +987,10 @@
         </is>
       </c>
       <c r="H10" t="n">
-        <v>45.45008657367337</v>
+        <v>45.39859105204894</v>
       </c>
       <c r="I10" t="n">
-        <v>12.36114426285248</v>
+        <v>12.3532020872167</v>
       </c>
       <c r="J10" t="inlineStr">
         <is>
@@ -1043,10 +1043,10 @@
         </is>
       </c>
       <c r="H11" t="n">
-        <v>45.55917093096186</v>
+        <v>45.56413567836782</v>
       </c>
       <c r="I11" t="n">
-        <v>11.55072115280037</v>
+        <v>11.54698172176243</v>
       </c>
       <c r="J11" t="inlineStr">
         <is>
@@ -1151,10 +1151,10 @@
         </is>
       </c>
       <c r="H13" t="n">
-        <v>45.51937686671877</v>
+        <v>45.51198118170051</v>
       </c>
       <c r="I13" t="n">
-        <v>11.58995559962064</v>
+        <v>11.54937540075043</v>
       </c>
       <c r="J13" t="inlineStr">
         <is>
@@ -1207,10 +1207,10 @@
         </is>
       </c>
       <c r="H14" t="n">
-        <v>45.57319720961723</v>
+        <v>45.5712410503055</v>
       </c>
       <c r="I14" t="n">
-        <v>11.54306723873088</v>
+        <v>11.54255823653188</v>
       </c>
       <c r="J14" t="inlineStr">
         <is>
@@ -1259,10 +1259,10 @@
         </is>
       </c>
       <c r="H15" t="n">
-        <v>45.41404808004538</v>
+        <v>45.37054234805176</v>
       </c>
       <c r="I15" t="n">
-        <v>11.9247422993236</v>
+        <v>11.90185411920182</v>
       </c>
       <c r="J15" t="inlineStr">
         <is>
@@ -1319,10 +1319,10 @@
         </is>
       </c>
       <c r="H16" t="n">
-        <v>45.55874450263094</v>
+        <v>45.59540516567597</v>
       </c>
       <c r="I16" t="n">
-        <v>11.5093386813512</v>
+        <v>11.56170727553564</v>
       </c>
       <c r="J16" t="inlineStr">
         <is>
@@ -1375,10 +1375,10 @@
         </is>
       </c>
       <c r="H17" t="n">
-        <v>45.5030332416044</v>
+        <v>45.53682668259852</v>
       </c>
       <c r="I17" t="n">
-        <v>11.58723045889424</v>
+        <v>11.50620100671729</v>
       </c>
       <c r="J17" t="inlineStr">
         <is>
@@ -1431,10 +1431,10 @@
         </is>
       </c>
       <c r="H18" t="n">
-        <v>45.58277364514104</v>
+        <v>45.57998327883453</v>
       </c>
       <c r="I18" t="n">
-        <v>11.50502588905754</v>
+        <v>11.5798464453228</v>
       </c>
       <c r="J18" t="inlineStr">
         <is>
@@ -1487,10 +1487,10 @@
         </is>
       </c>
       <c r="H19" t="n">
-        <v>45.53801425952619</v>
+        <v>45.5239010030983</v>
       </c>
       <c r="I19" t="n">
-        <v>11.49462393991348</v>
+        <v>11.52598429530358</v>
       </c>
       <c r="J19" t="inlineStr">
         <is>
@@ -1543,10 +1543,10 @@
         </is>
       </c>
       <c r="H20" t="n">
-        <v>45.52505921709245</v>
+        <v>45.51536076925926</v>
       </c>
       <c r="I20" t="n">
-        <v>11.55243291792553</v>
+        <v>11.5097741402916</v>
       </c>
       <c r="J20" t="inlineStr">
         <is>
@@ -1599,10 +1599,10 @@
         </is>
       </c>
       <c r="H21" t="n">
-        <v>45.55985125290867</v>
+        <v>45.52569963861534</v>
       </c>
       <c r="I21" t="n">
-        <v>11.54074429882253</v>
+        <v>11.55317328625458</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -1655,10 +1655,10 @@
         </is>
       </c>
       <c r="H22" t="n">
-        <v>45.57642700594123</v>
+        <v>45.51926084994588</v>
       </c>
       <c r="I22" t="n">
-        <v>11.56675161252684</v>
+        <v>11.59228741471364</v>
       </c>
       <c r="J22" t="inlineStr">
         <is>
@@ -1711,10 +1711,10 @@
         </is>
       </c>
       <c r="H23" t="n">
-        <v>45.53863294907438</v>
+        <v>45.54889467449403</v>
       </c>
       <c r="I23" t="n">
-        <v>11.57119480190919</v>
+        <v>11.53136438565799</v>
       </c>
       <c r="J23" t="inlineStr">
         <is>
@@ -1767,10 +1767,10 @@
         </is>
       </c>
       <c r="H24" t="n">
-        <v>45.37129541486311</v>
+        <v>45.3617966835512</v>
       </c>
       <c r="I24" t="n">
-        <v>11.860044767974</v>
+        <v>11.92244842967261</v>
       </c>
       <c r="J24" t="inlineStr">
         <is>
@@ -1827,10 +1827,10 @@
         </is>
       </c>
       <c r="H25" t="n">
-        <v>45.54414243342863</v>
+        <v>45.56976462330759</v>
       </c>
       <c r="I25" t="n">
-        <v>11.53276828289726</v>
+        <v>11.52305838545647</v>
       </c>
       <c r="J25" t="inlineStr">
         <is>
@@ -1887,10 +1887,10 @@
         </is>
       </c>
       <c r="H26" t="n">
-        <v>45.52430351804241</v>
+        <v>45.58787122665229</v>
       </c>
       <c r="I26" t="n">
-        <v>11.55828115240065</v>
+        <v>11.56635051870573</v>
       </c>
       <c r="J26" t="inlineStr">
         <is>
@@ -1947,10 +1947,10 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>45.37492790114071</v>
+        <v>45.39667096162415</v>
       </c>
       <c r="I27" t="n">
-        <v>11.82691807802824</v>
+        <v>11.91159743996491</v>
       </c>
       <c r="J27" t="inlineStr">
         <is>
@@ -2003,10 +2003,10 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>45.68294084471073</v>
+        <v>45.63465244819743</v>
       </c>
       <c r="I28" t="n">
-        <v>12.25560909936021</v>
+        <v>12.27304707059356</v>
       </c>
       <c r="J28" t="inlineStr">
         <is>
@@ -2059,10 +2059,10 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>45.47400698027393</v>
+        <v>45.45591464714174</v>
       </c>
       <c r="I29" t="n">
-        <v>12.30698681351336</v>
+        <v>12.27581224369264</v>
       </c>
       <c r="J29" t="inlineStr">
         <is>
@@ -2171,10 +2171,10 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>45.52644940622032</v>
+        <v>45.53288489399203</v>
       </c>
       <c r="I31" t="n">
-        <v>11.59176686930558</v>
+        <v>11.52509956452623</v>
       </c>
       <c r="J31" t="inlineStr">
         <is>
@@ -2283,10 +2283,10 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>45.58145562220422</v>
+        <v>45.53804902292848</v>
       </c>
       <c r="I33" t="n">
-        <v>11.55101744149068</v>
+        <v>11.51630340235046</v>
       </c>
       <c r="J33" t="inlineStr">
         <is>
@@ -2339,10 +2339,10 @@
         </is>
       </c>
       <c r="H34" t="n">
-        <v>45.39865283218138</v>
+        <v>45.36721287265154</v>
       </c>
       <c r="I34" t="n">
-        <v>11.91010713824587</v>
+        <v>11.84375631967432</v>
       </c>
       <c r="J34" t="inlineStr">
         <is>
@@ -2395,10 +2395,10 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>45.40664470889283</v>
+        <v>45.41516307424141</v>
       </c>
       <c r="I35" t="n">
-        <v>11.8841352993895</v>
+        <v>11.87425044468943</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
@@ -2451,10 +2451,10 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>45.38866602550757</v>
+        <v>45.39394350365104</v>
       </c>
       <c r="I36" t="n">
-        <v>11.88935191272723</v>
+        <v>11.86264944974869</v>
       </c>
       <c r="J36" t="inlineStr">
         <is>
@@ -2507,10 +2507,10 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>45.49969654953792</v>
+        <v>45.54888413735789</v>
       </c>
       <c r="I37" t="n">
-        <v>11.50156435153731</v>
+        <v>11.58651501284913</v>
       </c>
       <c r="J37" t="inlineStr">
         <is>
@@ -2563,10 +2563,10 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>45.56975191953734</v>
+        <v>45.53992413212389</v>
       </c>
       <c r="I38" t="n">
-        <v>11.49997013379913</v>
+        <v>11.50277486485785</v>
       </c>
       <c r="J38" t="inlineStr">
         <is>
@@ -2619,10 +2619,10 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>45.51780783240255</v>
+        <v>45.58182328369017</v>
       </c>
       <c r="I39" t="n">
-        <v>11.56617474817369</v>
+        <v>11.52371195226056</v>
       </c>
       <c r="J39" t="inlineStr">
         <is>
@@ -2675,10 +2675,10 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>45.59266578060734</v>
+        <v>45.54467157883811</v>
       </c>
       <c r="I40" t="n">
-        <v>11.58825300895093</v>
+        <v>11.51709928205664</v>
       </c>
       <c r="J40" t="inlineStr">
         <is>
@@ -2731,10 +2731,10 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>45.58740308961813</v>
+        <v>45.51508258367015</v>
       </c>
       <c r="I41" t="n">
-        <v>11.58230254357229</v>
+        <v>11.52575753088252</v>
       </c>
       <c r="J41" t="inlineStr">
         <is>
@@ -2787,10 +2787,10 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>45.42517168858602</v>
+        <v>45.38936975985517</v>
       </c>
       <c r="I42" t="n">
-        <v>11.90018879010626</v>
+        <v>11.89441625817105</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
@@ -2897,10 +2897,10 @@
         </is>
       </c>
       <c r="H44" t="n">
-        <v>45.55565265834315</v>
+        <v>45.59669172085987</v>
       </c>
       <c r="I44" t="n">
-        <v>11.51910724230643</v>
+        <v>11.49650043121449</v>
       </c>
       <c r="J44" t="inlineStr">
         <is>
@@ -2953,10 +2953,10 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>45.57587861895269</v>
+        <v>45.54414052677295</v>
       </c>
       <c r="I45" t="n">
-        <v>11.59119790606263</v>
+        <v>11.58004515545104</v>
       </c>
       <c r="J45" t="inlineStr">
         <is>
@@ -3009,10 +3009,10 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>45.4345329316907</v>
+        <v>45.39075596863377</v>
       </c>
       <c r="I46" t="n">
-        <v>11.87842172560638</v>
+        <v>11.84149615700036</v>
       </c>
       <c r="J46" t="inlineStr">
         <is>
@@ -3065,10 +3065,10 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>45.56830102561229</v>
+        <v>45.52041274911857</v>
       </c>
       <c r="I47" t="n">
-        <v>11.51905348519826</v>
+        <v>11.53536848969485</v>
       </c>
       <c r="J47" t="inlineStr">
         <is>
@@ -3125,10 +3125,10 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>45.564450087496</v>
+        <v>45.58575099037269</v>
       </c>
       <c r="I48" t="n">
-        <v>11.5201008846948</v>
+        <v>11.57257266055018</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -3181,10 +3181,10 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>45.51391912638272</v>
+        <v>45.52665888208475</v>
       </c>
       <c r="I49" t="n">
-        <v>11.50491176235838</v>
+        <v>11.50648397312396</v>
       </c>
       <c r="J49" t="inlineStr">
         <is>
@@ -3237,10 +3237,10 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>45.40456586325789</v>
+        <v>45.38579987747783</v>
       </c>
       <c r="I50" t="n">
-        <v>11.83189005219445</v>
+        <v>11.84016514249408</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -3295,10 +3295,10 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>45.55373788723878</v>
+        <v>45.51790769672546</v>
       </c>
       <c r="I51" t="n">
-        <v>11.510561968069</v>
+        <v>11.51525540342129</v>
       </c>
       <c r="J51" t="inlineStr">
         <is>
@@ -3351,10 +3351,10 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>45.50648981075519</v>
+        <v>45.52814238856895</v>
       </c>
       <c r="I52" t="n">
-        <v>11.57377768896716</v>
+        <v>11.49737834123315</v>
       </c>
       <c r="J52" t="inlineStr">
         <is>
@@ -3407,10 +3407,10 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>45.53446276722373</v>
+        <v>45.51307898108984</v>
       </c>
       <c r="I53" t="n">
-        <v>11.54426302761711</v>
+        <v>11.53098413860831</v>
       </c>
       <c r="J53" t="inlineStr">
         <is>
@@ -3467,10 +3467,10 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>45.50548124385413</v>
+        <v>45.52329375183771</v>
       </c>
       <c r="I54" t="n">
-        <v>11.55689803205049</v>
+        <v>11.54589144793436</v>
       </c>
       <c r="J54" t="inlineStr">
         <is>
@@ -3523,10 +3523,10 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>45.51828486451429</v>
+        <v>45.50433431452348</v>
       </c>
       <c r="I55" t="n">
-        <v>11.515011278414</v>
+        <v>11.5631631145361</v>
       </c>
       <c r="J55" t="inlineStr">
         <is>
@@ -3579,10 +3579,10 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>45.5874435854879</v>
+        <v>45.59114292707615</v>
       </c>
       <c r="I56" t="n">
-        <v>11.56975000258125</v>
+        <v>11.5026718458598</v>
       </c>
       <c r="J56" t="inlineStr">
         <is>
@@ -3635,10 +3635,10 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>45.5093065903624</v>
+        <v>45.54256338559654</v>
       </c>
       <c r="I57" t="n">
-        <v>11.51321768490096</v>
+        <v>11.55839856127538</v>
       </c>
       <c r="J57" t="inlineStr">
         <is>
@@ -3691,10 +3691,10 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>45.41891119894601</v>
+        <v>45.43105016742511</v>
       </c>
       <c r="I58" t="n">
-        <v>12.27373226299729</v>
+        <v>12.32583382319703</v>
       </c>
       <c r="J58" t="inlineStr">
         <is>
@@ -3747,10 +3747,10 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>45.50842620756818</v>
+        <v>45.56519491648769</v>
       </c>
       <c r="I59" t="n">
-        <v>11.57888756185503</v>
+        <v>11.57917755774779</v>
       </c>
       <c r="J59" t="inlineStr">
         <is>
@@ -3803,10 +3803,10 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>45.39733439008912</v>
+        <v>45.42952990740333</v>
       </c>
       <c r="I60" t="n">
-        <v>11.83578281201265</v>
+        <v>11.91123509694358</v>
       </c>
       <c r="J60" t="inlineStr">
         <is>
@@ -3963,10 +3963,10 @@
         </is>
       </c>
       <c r="H63" t="n">
-        <v>45.43274098754227</v>
+        <v>45.40308870504211</v>
       </c>
       <c r="I63" t="n">
-        <v>10.97523604746753</v>
+        <v>10.98586685441511</v>
       </c>
       <c r="J63" t="inlineStr">
         <is>
@@ -4019,10 +4019,10 @@
         </is>
       </c>
       <c r="H64" t="n">
-        <v>45.40578525190851</v>
+        <v>45.42380288192529</v>
       </c>
       <c r="I64" t="n">
-        <v>12.3472821907004</v>
+        <v>12.28248322139378</v>
       </c>
       <c r="J64" t="inlineStr">
         <is>
@@ -4075,10 +4075,10 @@
         </is>
       </c>
       <c r="H65" t="n">
-        <v>45.42060725400413</v>
+        <v>45.42694164462185</v>
       </c>
       <c r="I65" t="n">
-        <v>12.27741604244887</v>
+        <v>12.28219361867837</v>
       </c>
       <c r="J65" t="inlineStr">
         <is>
@@ -4131,10 +4131,10 @@
         </is>
       </c>
       <c r="H66" t="n">
-        <v>45.42135473197764</v>
+        <v>45.38930900414127</v>
       </c>
       <c r="I66" t="n">
-        <v>10.97852578049745</v>
+        <v>10.97406401089688</v>
       </c>
       <c r="J66" t="inlineStr">
         <is>
@@ -4187,10 +4187,10 @@
         </is>
       </c>
       <c r="H67" t="n">
-        <v>45.39058377478719</v>
+        <v>45.45205803343016</v>
       </c>
       <c r="I67" t="n">
-        <v>11.91829721615317</v>
+        <v>11.87820014212608</v>
       </c>
       <c r="J67" t="inlineStr">
         <is>
@@ -4243,10 +4243,10 @@
         </is>
       </c>
       <c r="H68" t="n">
-        <v>45.58264450372386</v>
+        <v>45.52378801901811</v>
       </c>
       <c r="I68" t="n">
-        <v>11.51195216697314</v>
+        <v>11.57742393023254</v>
       </c>
       <c r="J68" t="inlineStr">
         <is>
@@ -4299,10 +4299,10 @@
         </is>
       </c>
       <c r="H69" t="n">
-        <v>45.55560434003141</v>
+        <v>45.57577403650354</v>
       </c>
       <c r="I69" t="n">
-        <v>11.53680772252439</v>
+        <v>11.5787075445803</v>
       </c>
       <c r="J69" t="inlineStr">
         <is>
@@ -4355,10 +4355,10 @@
         </is>
       </c>
       <c r="H70" t="n">
-        <v>45.54145595553196</v>
+        <v>45.50045591691055</v>
       </c>
       <c r="I70" t="n">
-        <v>11.49684725624359</v>
+        <v>11.56383133359826</v>
       </c>
       <c r="J70" t="inlineStr">
         <is>
@@ -4411,10 +4411,10 @@
         </is>
       </c>
       <c r="H71" t="n">
-        <v>45.50789205818558</v>
+        <v>45.54095822100361</v>
       </c>
       <c r="I71" t="n">
-        <v>11.56926357041898</v>
+        <v>11.59165531798094</v>
       </c>
       <c r="J71" t="inlineStr">
         <is>
@@ -4467,10 +4467,10 @@
         </is>
       </c>
       <c r="H72" t="n">
-        <v>45.5029660881636</v>
+        <v>45.5901846688996</v>
       </c>
       <c r="I72" t="n">
-        <v>11.5566889083416</v>
+        <v>11.57861466363811</v>
       </c>
       <c r="J72" t="inlineStr">
         <is>
@@ -4523,10 +4523,10 @@
         </is>
       </c>
       <c r="H73" t="n">
-        <v>45.52851641571593</v>
+        <v>45.58599235272514</v>
       </c>
       <c r="I73" t="n">
-        <v>11.57039489634427</v>
+        <v>11.58918467866261</v>
       </c>
       <c r="J73" t="inlineStr">
         <is>
@@ -4579,10 +4579,10 @@
         </is>
       </c>
       <c r="H74" t="n">
-        <v>45.55339588149291</v>
+        <v>45.56355682123213</v>
       </c>
       <c r="I74" t="n">
-        <v>11.54148590574642</v>
+        <v>11.52166304626273</v>
       </c>
       <c r="J74" t="inlineStr">
         <is>
@@ -4635,10 +4635,10 @@
         </is>
       </c>
       <c r="H75" t="n">
-        <v>45.50428517549039</v>
+        <v>45.55018669044272</v>
       </c>
       <c r="I75" t="n">
-        <v>11.58318191003318</v>
+        <v>11.56149794995895</v>
       </c>
       <c r="J75" t="inlineStr">
         <is>
@@ -4691,10 +4691,10 @@
         </is>
       </c>
       <c r="H76" t="n">
-        <v>45.52392411906253</v>
+        <v>45.54960242251548</v>
       </c>
       <c r="I76" t="n">
-        <v>11.4985789487193</v>
+        <v>11.56271612215622</v>
       </c>
       <c r="J76" t="inlineStr">
         <is>
@@ -4747,10 +4747,10 @@
         </is>
       </c>
       <c r="H77" t="n">
-        <v>45.41813477141283</v>
+        <v>45.40612651366183</v>
       </c>
       <c r="I77" t="n">
-        <v>12.28223417582515</v>
+        <v>12.31166017512852</v>
       </c>
       <c r="J77" t="inlineStr">
         <is>
@@ -4803,10 +4803,10 @@
         </is>
       </c>
       <c r="H78" t="n">
-        <v>45.45241836332138</v>
+        <v>45.43147482259386</v>
       </c>
       <c r="I78" t="n">
-        <v>11.91490298108437</v>
+        <v>11.86090314639996</v>
       </c>
       <c r="J78" t="inlineStr">
         <is>
@@ -4859,10 +4859,10 @@
         </is>
       </c>
       <c r="H79" t="n">
-        <v>45.39748276929736</v>
+        <v>45.36139842697055</v>
       </c>
       <c r="I79" t="n">
-        <v>11.84645818872833</v>
+        <v>11.8377090502165</v>
       </c>
       <c r="J79" t="inlineStr">
         <is>
@@ -4917,10 +4917,10 @@
         </is>
       </c>
       <c r="H80" t="n">
-        <v>45.37316404255913</v>
+        <v>45.44745602867025</v>
       </c>
       <c r="I80" t="n">
-        <v>11.88234948898527</v>
+        <v>11.92454294339201</v>
       </c>
       <c r="J80" t="inlineStr">
         <is>
@@ -4973,10 +4973,10 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>45.58252408004147</v>
+        <v>45.4997706277453</v>
       </c>
       <c r="I81" t="n">
-        <v>11.50219522142386</v>
+        <v>11.52694892750597</v>
       </c>
       <c r="J81" t="inlineStr">
         <is>
@@ -5029,10 +5029,10 @@
         </is>
       </c>
       <c r="H82" t="n">
-        <v>45.5532260923673</v>
+        <v>45.56497222237699</v>
       </c>
       <c r="I82" t="n">
-        <v>11.59180097368953</v>
+        <v>11.54143916986996</v>
       </c>
       <c r="J82" t="inlineStr">
         <is>
@@ -5087,10 +5087,10 @@
         </is>
       </c>
       <c r="H83" t="n">
-        <v>45.41595279467352</v>
+        <v>45.37423704006719</v>
       </c>
       <c r="I83" t="n">
-        <v>11.82762967062275</v>
+        <v>11.82767453238398</v>
       </c>
       <c r="J83" t="inlineStr">
         <is>
@@ -5143,10 +5143,10 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>45.58352699377387</v>
+        <v>45.51497076419402</v>
       </c>
       <c r="I84" t="n">
-        <v>11.54826763192349</v>
+        <v>11.57250994482773</v>
       </c>
       <c r="J84" t="inlineStr">
         <is>
@@ -5199,10 +5199,10 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>45.41742105995576</v>
+        <v>45.43585302075641</v>
       </c>
       <c r="I85" t="n">
-        <v>12.34550350564168</v>
+        <v>12.26722122729284</v>
       </c>
       <c r="J85" t="inlineStr">
         <is>
@@ -5255,10 +5255,10 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>45.58434404312744</v>
+        <v>45.52854833363518</v>
       </c>
       <c r="I86" t="n">
-        <v>11.52538887709408</v>
+        <v>11.57356709969397</v>
       </c>
       <c r="J86" t="inlineStr">
         <is>
@@ -5311,10 +5311,10 @@
         </is>
       </c>
       <c r="H87" t="n">
-        <v>45.57083515765471</v>
+        <v>45.59715572372757</v>
       </c>
       <c r="I87" t="n">
-        <v>11.51283969219926</v>
+        <v>11.5730068754176</v>
       </c>
       <c r="J87" t="inlineStr">
         <is>
@@ -5367,10 +5367,10 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>45.40534588154664</v>
+        <v>45.43959182252329</v>
       </c>
       <c r="I88" t="n">
-        <v>12.31194534803803</v>
+        <v>12.3179044863</v>
       </c>
       <c r="J88" t="inlineStr">
         <is>
@@ -5423,10 +5423,10 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>45.37157916634606</v>
+        <v>45.42873685968549</v>
       </c>
       <c r="I89" t="n">
-        <v>11.86879624141607</v>
+        <v>11.84758910996072</v>
       </c>
       <c r="J89" t="inlineStr">
         <is>
@@ -5479,10 +5479,10 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>45.39468859704859</v>
+        <v>45.40196583855953</v>
       </c>
       <c r="I90" t="n">
-        <v>11.85302212389705</v>
+        <v>11.86824533366205</v>
       </c>
       <c r="J90" t="inlineStr">
         <is>
@@ -5535,10 +5535,10 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>45.59046910542991</v>
+        <v>45.55174557450274</v>
       </c>
       <c r="I91" t="n">
-        <v>11.53641902676103</v>
+        <v>11.53094103129491</v>
       </c>
       <c r="J91" t="inlineStr">
         <is>
@@ -5591,10 +5591,10 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>45.54911848324085</v>
+        <v>45.51608525532363</v>
       </c>
       <c r="I92" t="n">
-        <v>11.53215231335692</v>
+        <v>11.54590241235254</v>
       </c>
       <c r="J92" t="inlineStr">
         <is>
@@ -5647,10 +5647,10 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>45.58453615503126</v>
+        <v>45.5333811305433</v>
       </c>
       <c r="I93" t="n">
-        <v>11.51854037278972</v>
+        <v>11.51447808121686</v>
       </c>
       <c r="J93" t="inlineStr">
         <is>
@@ -5703,10 +5703,10 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>45.44405418595409</v>
+        <v>45.44835283034138</v>
       </c>
       <c r="I94" t="n">
-        <v>11.89588065936301</v>
+        <v>11.92243765397179</v>
       </c>
       <c r="J94" t="inlineStr">
         <is>
@@ -5759,10 +5759,10 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>45.45035031208563</v>
+        <v>45.42304829421111</v>
       </c>
       <c r="I95" t="n">
-        <v>11.92022611443391</v>
+        <v>11.84750489957948</v>
       </c>
       <c r="J95" t="inlineStr">
         <is>
@@ -5815,10 +5815,10 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>45.46019300978714</v>
+        <v>45.48317031501985</v>
       </c>
       <c r="I96" t="n">
-        <v>12.28843324928426</v>
+        <v>12.31988741296238</v>
       </c>
       <c r="J96" t="inlineStr">
         <is>
@@ -5871,10 +5871,10 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>45.5339641389695</v>
+        <v>45.5146141116312</v>
       </c>
       <c r="I97" t="n">
-        <v>11.5629679471752</v>
+        <v>11.53149917285251</v>
       </c>
       <c r="J97" t="inlineStr">
         <is>
@@ -5927,10 +5927,10 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>45.51106608149315</v>
+        <v>45.51186376173073</v>
       </c>
       <c r="I98" t="n">
-        <v>11.55682579441374</v>
+        <v>11.57539846308679</v>
       </c>
       <c r="J98" t="inlineStr">
         <is>
@@ -5983,10 +5983,10 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>45.53409642238957</v>
+        <v>45.49791350926126</v>
       </c>
       <c r="I99" t="n">
-        <v>11.49673947011571</v>
+        <v>11.58842506535872</v>
       </c>
       <c r="J99" t="inlineStr">
         <is>
@@ -6039,10 +6039,10 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>45.59646276466043</v>
+        <v>45.54389862131126</v>
       </c>
       <c r="I100" t="n">
-        <v>11.52619964448511</v>
+        <v>11.56998441542495</v>
       </c>
       <c r="J100" t="inlineStr">
         <is>
@@ -6095,10 +6095,10 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>45.58147765102416</v>
+        <v>45.50950107680003</v>
       </c>
       <c r="I101" t="n">
-        <v>11.49529224443035</v>
+        <v>11.50215909308355</v>
       </c>
       <c r="J101" t="inlineStr">
         <is>
@@ -6151,10 +6151,10 @@
         </is>
       </c>
       <c r="H102" t="n">
-        <v>45.57450198183881</v>
+        <v>45.55446783215851</v>
       </c>
       <c r="I102" t="n">
-        <v>11.55589858367643</v>
+        <v>11.51862951472959</v>
       </c>
       <c r="J102" t="inlineStr">
         <is>
@@ -6207,10 +6207,10 @@
         </is>
       </c>
       <c r="H103" t="n">
-        <v>45.43422487720012</v>
+        <v>45.38451448516841</v>
       </c>
       <c r="I103" t="n">
-        <v>11.8594809273083</v>
+        <v>11.82817188506748</v>
       </c>
       <c r="J103" t="inlineStr">
         <is>
@@ -6263,10 +6263,10 @@
         </is>
       </c>
       <c r="H104" t="n">
-        <v>45.53264363440219</v>
+        <v>45.58643860728831</v>
       </c>
       <c r="I104" t="n">
-        <v>11.54009109513898</v>
+        <v>11.56393229465978</v>
       </c>
       <c r="J104" t="inlineStr">
         <is>
@@ -6319,10 +6319,10 @@
         </is>
       </c>
       <c r="H105" t="n">
-        <v>45.56477527508265</v>
+        <v>45.51821713966697</v>
       </c>
       <c r="I105" t="n">
-        <v>11.53509818371972</v>
+        <v>11.57234478974233</v>
       </c>
       <c r="J105" t="inlineStr">
         <is>
@@ -6375,10 +6375,10 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>45.62940702333776</v>
+        <v>45.66254093204451</v>
       </c>
       <c r="I106" t="n">
-        <v>12.22032757736011</v>
+        <v>12.2385523530891</v>
       </c>
       <c r="J106" t="inlineStr">
         <is>
@@ -6431,10 +6431,10 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>45.57017153300971</v>
+        <v>45.51665388294887</v>
       </c>
       <c r="I107" t="n">
-        <v>11.59077750989782</v>
+        <v>11.55385667567973</v>
       </c>
       <c r="J107" t="inlineStr">
         <is>
@@ -6487,10 +6487,10 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>45.58533077688097</v>
+        <v>45.56974544881707</v>
       </c>
       <c r="I108" t="n">
-        <v>11.53377888981069</v>
+        <v>11.58194309545047</v>
       </c>
       <c r="J108" t="inlineStr">
         <is>
@@ -6543,10 +6543,10 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>45.59706168321733</v>
+        <v>45.53819021566494</v>
       </c>
       <c r="I109" t="n">
-        <v>11.59316304965835</v>
+        <v>11.51548237581501</v>
       </c>
       <c r="J109" t="inlineStr">
         <is>
@@ -6599,10 +6599,10 @@
         </is>
       </c>
       <c r="H110" t="n">
-        <v>45.43272288185121</v>
+        <v>45.40118148892511</v>
       </c>
       <c r="I110" t="n">
-        <v>11.88277407546876</v>
+        <v>11.84671028306105</v>
       </c>
       <c r="J110" t="inlineStr">
         <is>
@@ -6655,10 +6655,10 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>45.5746896359239</v>
+        <v>45.54809943011527</v>
       </c>
       <c r="I111" t="n">
-        <v>11.53731940260658</v>
+        <v>11.57683884371839</v>
       </c>
       <c r="J111" t="inlineStr">
         <is>
@@ -6711,10 +6711,10 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>45.40245544383298</v>
+        <v>45.38272241765974</v>
       </c>
       <c r="I112" t="n">
-        <v>11.88628975595158</v>
+        <v>11.84179257420525</v>
       </c>
       <c r="J112" t="inlineStr">
         <is>
@@ -6767,10 +6767,10 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>45.40285116241176</v>
+        <v>45.40819289189341</v>
       </c>
       <c r="I113" t="n">
-        <v>11.91385111880946</v>
+        <v>11.8581880857476</v>
       </c>
       <c r="J113" t="inlineStr">
         <is>
@@ -6823,10 +6823,10 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>45.42052428693763</v>
+        <v>45.48481008720231</v>
       </c>
       <c r="I114" t="n">
-        <v>11.03775847770881</v>
+        <v>10.98814689998412</v>
       </c>
       <c r="J114" t="inlineStr">
         <is>
@@ -6931,10 +6931,10 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>45.44959722939014</v>
+        <v>45.38046194316956</v>
       </c>
       <c r="I116" t="n">
-        <v>11.84725579005288</v>
+        <v>11.85802061738671</v>
       </c>
       <c r="J116" t="inlineStr">
         <is>
@@ -6987,10 +6987,10 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>45.53544413436089</v>
+        <v>45.52239118312987</v>
       </c>
       <c r="I117" t="n">
-        <v>11.54132217945515</v>
+        <v>11.54902184090547</v>
       </c>
       <c r="J117" t="inlineStr">
         <is>
@@ -7043,10 +7043,10 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>45.59031525653277</v>
+        <v>45.53772515861009</v>
       </c>
       <c r="I118" t="n">
-        <v>11.52844355483706</v>
+        <v>11.52905728721917</v>
       </c>
       <c r="J118" t="inlineStr">
         <is>
@@ -7099,10 +7099,10 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>45.44454803512401</v>
+        <v>45.4158521682992</v>
       </c>
       <c r="I119" t="n">
-        <v>11.82934407155218</v>
+        <v>11.86375914111254</v>
       </c>
       <c r="J119" t="inlineStr">
         <is>
@@ -7155,10 +7155,10 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>45.37350519217143</v>
+        <v>45.36155883715509</v>
       </c>
       <c r="I120" t="n">
-        <v>11.88165763610416</v>
+        <v>11.85889753720416</v>
       </c>
       <c r="J120" t="inlineStr">
         <is>
@@ -7211,10 +7211,10 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>45.5455816474307</v>
+        <v>45.58011509471896</v>
       </c>
       <c r="I121" t="n">
-        <v>11.5061147104664</v>
+        <v>11.5448730768351</v>
       </c>
       <c r="J121" t="inlineStr">
         <is>
@@ -7267,10 +7267,10 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>45.54038383169075</v>
+        <v>45.5666796483541</v>
       </c>
       <c r="I122" t="n">
-        <v>11.55424277798868</v>
+        <v>11.54472403837381</v>
       </c>
       <c r="J122" t="inlineStr">
         <is>
@@ -7323,10 +7323,10 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>45.52457294168251</v>
+        <v>45.5041589550561</v>
       </c>
       <c r="I123" t="n">
-        <v>11.59298869721716</v>
+        <v>11.50582325474111</v>
       </c>
       <c r="J123" t="inlineStr">
         <is>
@@ -7379,10 +7379,10 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>45.58259703024723</v>
+        <v>45.5681828519746</v>
       </c>
       <c r="I124" t="n">
-        <v>11.56585168110529</v>
+        <v>11.52816242653823</v>
       </c>
       <c r="J124" t="inlineStr">
         <is>
@@ -7435,10 +7435,10 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>45.4341996064879</v>
+        <v>45.42664785336429</v>
       </c>
       <c r="I125" t="n">
-        <v>11.84307647671988</v>
+        <v>11.91403182923532</v>
       </c>
       <c r="J125" t="inlineStr">
         <is>
@@ -7491,10 +7491,10 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>45.44846057493338</v>
+        <v>45.37844718802308</v>
       </c>
       <c r="I126" t="n">
-        <v>11.90808085397519</v>
+        <v>11.83567310905736</v>
       </c>
       <c r="J126" t="inlineStr">
         <is>
@@ -7547,10 +7547,10 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>45.39288775851406</v>
+        <v>45.44393362068354</v>
       </c>
       <c r="I127" t="n">
-        <v>12.3536192574267</v>
+        <v>12.31915966067802</v>
       </c>
       <c r="J127" t="inlineStr">
         <is>
@@ -7603,10 +7603,10 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>45.53140861958466</v>
+        <v>45.56848977240485</v>
       </c>
       <c r="I128" t="n">
-        <v>11.50098609549167</v>
+        <v>11.57623084289722</v>
       </c>
       <c r="J128" t="inlineStr">
         <is>
@@ -7659,10 +7659,10 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>45.35821853971531</v>
+        <v>45.38908167938936</v>
       </c>
       <c r="I129" t="n">
-        <v>11.86757375377814</v>
+        <v>11.83001589199794</v>
       </c>
       <c r="J129" t="inlineStr">
         <is>
@@ -7715,10 +7715,10 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>45.40083871959532</v>
+        <v>45.42014239596796</v>
       </c>
       <c r="I130" t="n">
-        <v>11.90814251616833</v>
+        <v>11.89385266249748</v>
       </c>
       <c r="J130" t="inlineStr">
         <is>
@@ -7771,10 +7771,10 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>45.6780524903977</v>
+        <v>45.6745541192682</v>
       </c>
       <c r="I131" t="n">
-        <v>12.21057158096952</v>
+        <v>12.29198290044885</v>
       </c>
       <c r="J131" t="inlineStr">
         <is>
@@ -7827,10 +7827,10 @@
         </is>
       </c>
       <c r="H132" t="n">
-        <v>45.48883147206575</v>
+        <v>45.46015943912038</v>
       </c>
       <c r="I132" t="n">
-        <v>12.36509520591687</v>
+        <v>12.33641917456987</v>
       </c>
       <c r="J132" t="inlineStr">
         <is>
@@ -7883,10 +7883,10 @@
         </is>
       </c>
       <c r="H133" t="n">
-        <v>45.57890845963126</v>
+        <v>45.49881409792306</v>
       </c>
       <c r="I133" t="n">
-        <v>11.58113265335724</v>
+        <v>11.51656184142672</v>
       </c>
       <c r="J133" t="inlineStr">
         <is>
@@ -7939,10 +7939,10 @@
         </is>
       </c>
       <c r="H134" t="n">
-        <v>45.43608487236583</v>
+        <v>45.42712239148255</v>
       </c>
       <c r="I134" t="n">
-        <v>11.82688072490648</v>
+        <v>11.86592800307823</v>
       </c>
       <c r="J134" t="inlineStr">
         <is>
@@ -8043,10 +8043,10 @@
         </is>
       </c>
       <c r="H136" t="n">
-        <v>45.36075230806144</v>
+        <v>45.4445237071977</v>
       </c>
       <c r="I136" t="n">
-        <v>11.87526349911749</v>
+        <v>11.85671872969671</v>
       </c>
       <c r="J136" t="inlineStr">
         <is>
@@ -8099,10 +8099,10 @@
         </is>
       </c>
       <c r="H137" t="n">
-        <v>45.51793355259426</v>
+        <v>45.51535161719262</v>
       </c>
       <c r="I137" t="n">
-        <v>11.54076471412693</v>
+        <v>11.52024526368519</v>
       </c>
       <c r="J137" t="inlineStr">
         <is>
@@ -8155,10 +8155,10 @@
         </is>
       </c>
       <c r="H138" t="n">
-        <v>45.50427455019116</v>
+        <v>45.52420743431706</v>
       </c>
       <c r="I138" t="n">
-        <v>11.58229240915701</v>
+        <v>11.5523522501763</v>
       </c>
       <c r="J138" t="inlineStr">
         <is>
@@ -8211,10 +8211,10 @@
         </is>
       </c>
       <c r="H139" t="n">
-        <v>45.5808732207062</v>
+        <v>45.58853671951663</v>
       </c>
       <c r="I139" t="n">
-        <v>11.4996842030352</v>
+        <v>11.59265455344492</v>
       </c>
       <c r="J139" t="inlineStr">
         <is>
@@ -8267,10 +8267,10 @@
         </is>
       </c>
       <c r="H140" t="n">
-        <v>45.39117041527486</v>
+        <v>45.47407764998237</v>
       </c>
       <c r="I140" t="n">
-        <v>12.30218035609782</v>
+        <v>12.2859919103136</v>
       </c>
       <c r="J140" t="inlineStr">
         <is>
@@ -8323,10 +8323,10 @@
         </is>
       </c>
       <c r="H141" t="n">
-        <v>45.41852588316912</v>
+        <v>45.47979208641413</v>
       </c>
       <c r="I141" t="n">
-        <v>12.34755179291434</v>
+        <v>12.26883471242774</v>
       </c>
       <c r="J141" t="inlineStr">
         <is>
@@ -8427,10 +8427,10 @@
         </is>
       </c>
       <c r="H143" t="n">
-        <v>45.52161004541721</v>
+        <v>45.51220328928375</v>
       </c>
       <c r="I143" t="n">
-        <v>11.54986598687713</v>
+        <v>11.55660506200705</v>
       </c>
       <c r="J143" t="inlineStr">
         <is>
@@ -8483,10 +8483,10 @@
         </is>
       </c>
       <c r="H144" t="n">
-        <v>45.55708081646969</v>
+        <v>45.55222714710217</v>
       </c>
       <c r="I144" t="n">
-        <v>11.53627245490078</v>
+        <v>11.55627312682076</v>
       </c>
       <c r="J144" t="inlineStr">
         <is>
@@ -8539,10 +8539,10 @@
         </is>
       </c>
       <c r="H145" t="n">
-        <v>45.5522646848472</v>
+        <v>45.50693417103908</v>
       </c>
       <c r="I145" t="n">
-        <v>11.5382514696044</v>
+        <v>11.54098235242515</v>
       </c>
       <c r="J145" t="inlineStr">
         <is>
@@ -8595,10 +8595,10 @@
         </is>
       </c>
       <c r="H146" t="n">
-        <v>45.52099375849014</v>
+        <v>45.50988577066824</v>
       </c>
       <c r="I146" t="n">
-        <v>11.52938709895235</v>
+        <v>11.50601159771644</v>
       </c>
       <c r="J146" t="inlineStr">
         <is>
@@ -8651,10 +8651,10 @@
         </is>
       </c>
       <c r="H147" t="n">
-        <v>45.572186135889</v>
+        <v>45.59142773218514</v>
       </c>
       <c r="I147" t="n">
-        <v>11.52116658596029</v>
+        <v>11.59120211305772</v>
       </c>
       <c r="J147" t="inlineStr">
         <is>
@@ -8707,10 +8707,10 @@
         </is>
       </c>
       <c r="H148" t="n">
-        <v>45.57613810577075</v>
+        <v>45.5241334619926</v>
       </c>
       <c r="I148" t="n">
-        <v>11.53938181940718</v>
+        <v>11.54865246421715</v>
       </c>
       <c r="J148" t="inlineStr">
         <is>
@@ -8759,10 +8759,10 @@
         </is>
       </c>
       <c r="H149" t="n">
-        <v>45.50803407732109</v>
+        <v>45.5166015781036</v>
       </c>
       <c r="I149" t="n">
-        <v>11.52783134138812</v>
+        <v>11.52345682986263</v>
       </c>
       <c r="J149" t="inlineStr">
         <is>
@@ -8815,10 +8815,10 @@
         </is>
       </c>
       <c r="H150" t="n">
-        <v>45.542245425304</v>
+        <v>45.56645550353142</v>
       </c>
       <c r="I150" t="n">
-        <v>11.52261780044995</v>
+        <v>11.55748381427141</v>
       </c>
       <c r="J150" t="inlineStr">
         <is>
@@ -8871,10 +8871,10 @@
         </is>
       </c>
       <c r="H151" t="n">
-        <v>45.51644176291619</v>
+        <v>45.57808015857194</v>
       </c>
       <c r="I151" t="n">
-        <v>11.56737734417882</v>
+        <v>11.58302966671427</v>
       </c>
       <c r="J151" t="inlineStr">
         <is>
@@ -8927,10 +8927,10 @@
         </is>
       </c>
       <c r="H152" t="n">
-        <v>45.53242230882297</v>
+        <v>45.58534688276326</v>
       </c>
       <c r="I152" t="n">
-        <v>11.51818069656486</v>
+        <v>11.53842683276861</v>
       </c>
       <c r="J152" t="inlineStr">
         <is>
@@ -8983,10 +8983,10 @@
         </is>
       </c>
       <c r="H153" t="n">
-        <v>45.50827149157359</v>
+        <v>45.5318510500416</v>
       </c>
       <c r="I153" t="n">
-        <v>11.49930343134439</v>
+        <v>11.58365646294399</v>
       </c>
       <c r="J153" t="inlineStr">
         <is>
@@ -9039,10 +9039,10 @@
         </is>
       </c>
       <c r="H154" t="n">
-        <v>45.54807611657569</v>
+        <v>45.54357922582794</v>
       </c>
       <c r="I154" t="n">
-        <v>11.53643511828528</v>
+        <v>11.53955014231866</v>
       </c>
       <c r="J154" t="inlineStr">
         <is>
@@ -9095,10 +9095,10 @@
         </is>
       </c>
       <c r="H155" t="n">
-        <v>45.40324309141933</v>
+        <v>45.42998164223241</v>
       </c>
       <c r="I155" t="n">
-        <v>11.85773500581337</v>
+        <v>11.84112385994592</v>
       </c>
       <c r="J155" t="inlineStr">
         <is>
@@ -9151,10 +9151,10 @@
         </is>
       </c>
       <c r="H156" t="n">
-        <v>45.45025044150962</v>
+        <v>45.44749418180777</v>
       </c>
       <c r="I156" t="n">
-        <v>12.32256739892571</v>
+        <v>12.33631877270279</v>
       </c>
       <c r="J156" t="inlineStr">
         <is>
@@ -9207,10 +9207,10 @@
         </is>
       </c>
       <c r="H157" t="n">
-        <v>45.53158109933202</v>
+        <v>45.58843901976524</v>
       </c>
       <c r="I157" t="n">
-        <v>11.58906926465416</v>
+        <v>11.49892966428809</v>
       </c>
       <c r="J157" t="inlineStr">
         <is>
@@ -9315,10 +9315,10 @@
         </is>
       </c>
       <c r="H159" t="n">
-        <v>45.40861720476087</v>
+        <v>45.39998795707997</v>
       </c>
       <c r="I159" t="n">
-        <v>11.84207262997222</v>
+        <v>11.90394689387699</v>
       </c>
       <c r="J159" t="inlineStr">
         <is>
@@ -9371,10 +9371,10 @@
         </is>
       </c>
       <c r="H160" t="n">
-        <v>45.69458859446611</v>
+        <v>45.64361918503048</v>
       </c>
       <c r="I160" t="n">
-        <v>12.27489436554277</v>
+        <v>12.22173189966023</v>
       </c>
       <c r="J160" t="inlineStr">
         <is>
@@ -9427,10 +9427,10 @@
         </is>
       </c>
       <c r="H161" t="n">
-        <v>45.38302667850173</v>
+        <v>45.4491118194716</v>
       </c>
       <c r="I161" t="n">
-        <v>11.84181731551589</v>
+        <v>11.82997815254211</v>
       </c>
       <c r="J161" t="inlineStr">
         <is>
@@ -9479,10 +9479,10 @@
         </is>
       </c>
       <c r="H162" t="n">
-        <v>45.55916112691272</v>
+        <v>45.58503404463162</v>
       </c>
       <c r="I162" t="n">
-        <v>11.56697918448907</v>
+        <v>11.5022820828739</v>
       </c>
       <c r="J162" t="inlineStr">
         <is>
@@ -9535,10 +9535,10 @@
         </is>
       </c>
       <c r="H163" t="n">
-        <v>45.50654518443515</v>
+        <v>45.53558077848894</v>
       </c>
       <c r="I163" t="n">
-        <v>11.50590576390129</v>
+        <v>11.5605563565554</v>
       </c>
       <c r="J163" t="inlineStr">
         <is>
@@ -9591,10 +9591,10 @@
         </is>
       </c>
       <c r="H164" t="n">
-        <v>45.5562033592207</v>
+        <v>45.59264418649945</v>
       </c>
       <c r="I164" t="n">
-        <v>11.57743178602216</v>
+        <v>11.53786022437725</v>
       </c>
       <c r="J164" t="inlineStr">
         <is>
@@ -9651,10 +9651,10 @@
         </is>
       </c>
       <c r="H165" t="n">
-        <v>45.42065736818013</v>
+        <v>45.41177976125962</v>
       </c>
       <c r="I165" t="n">
-        <v>11.85494022051201</v>
+        <v>11.85187537330898</v>
       </c>
       <c r="J165" t="inlineStr">
         <is>
@@ -9707,10 +9707,10 @@
         </is>
       </c>
       <c r="H166" t="n">
-        <v>45.5344377279448</v>
+        <v>45.53679341495733</v>
       </c>
       <c r="I166" t="n">
-        <v>11.49754295656469</v>
+        <v>11.57823820984</v>
       </c>
       <c r="J166" t="inlineStr">
         <is>
@@ -9763,10 +9763,10 @@
         </is>
       </c>
       <c r="H167" t="n">
-        <v>45.71079318614279</v>
+        <v>45.68689289207688</v>
       </c>
       <c r="I167" t="n">
-        <v>12.26308179157376</v>
+        <v>12.25452971378449</v>
       </c>
       <c r="J167" t="inlineStr">
         <is>
@@ -9819,10 +9819,10 @@
         </is>
       </c>
       <c r="H168" t="n">
-        <v>45.59662286789622</v>
+        <v>45.58567549298108</v>
       </c>
       <c r="I168" t="n">
-        <v>11.53374640913669</v>
+        <v>11.53799344066115</v>
       </c>
       <c r="J168" t="inlineStr">
         <is>
@@ -9875,10 +9875,10 @@
         </is>
       </c>
       <c r="H169" t="n">
-        <v>45.39322079394877</v>
+        <v>45.43633152943838</v>
       </c>
       <c r="I169" t="n">
-        <v>11.83339636560445</v>
+        <v>11.89702888263338</v>
       </c>
       <c r="J169" t="inlineStr">
         <is>
@@ -9931,10 +9931,10 @@
         </is>
       </c>
       <c r="H170" t="n">
-        <v>45.71668310251989</v>
+        <v>45.69526461575903</v>
       </c>
       <c r="I170" t="n">
-        <v>12.2689346636618</v>
+        <v>12.22465475670767</v>
       </c>
       <c r="J170" t="inlineStr">
         <is>
@@ -9987,10 +9987,10 @@
         </is>
       </c>
       <c r="H171" t="n">
-        <v>45.38888828446867</v>
+        <v>45.48603222230834</v>
       </c>
       <c r="I171" t="n">
-        <v>11.02767151966088</v>
+        <v>10.98140652934045</v>
       </c>
       <c r="J171" t="inlineStr">
         <is>
@@ -10043,10 +10043,10 @@
         </is>
       </c>
       <c r="H172" t="n">
-        <v>45.54372886555554</v>
+        <v>45.57901229722267</v>
       </c>
       <c r="I172" t="n">
-        <v>11.58616267498932</v>
+        <v>11.58115069547673</v>
       </c>
       <c r="J172" t="inlineStr">
         <is>
@@ -10099,10 +10099,10 @@
         </is>
       </c>
       <c r="H173" t="n">
-        <v>45.53975433667028</v>
+        <v>45.52286834583753</v>
       </c>
       <c r="I173" t="n">
-        <v>11.55303620607196</v>
+        <v>11.54377802165451</v>
       </c>
       <c r="J173" t="inlineStr">
         <is>
@@ -10155,10 +10155,10 @@
         </is>
       </c>
       <c r="H174" t="n">
-        <v>45.53382921669539</v>
+        <v>45.59616369513132</v>
       </c>
       <c r="I174" t="n">
-        <v>11.55003207338631</v>
+        <v>11.58976636553671</v>
       </c>
       <c r="J174" t="inlineStr">
         <is>
@@ -10211,10 +10211,10 @@
         </is>
       </c>
       <c r="H175" t="n">
-        <v>45.63422273375438</v>
+        <v>45.66067960555407</v>
       </c>
       <c r="I175" t="n">
-        <v>12.23087480614655</v>
+        <v>12.21334047145831</v>
       </c>
       <c r="J175" t="inlineStr">
         <is>
@@ -10267,10 +10267,10 @@
         </is>
       </c>
       <c r="H176" t="n">
-        <v>45.5718669017446</v>
+        <v>45.56558876744622</v>
       </c>
       <c r="I176" t="n">
-        <v>11.57696858389577</v>
+        <v>11.50983159070421</v>
       </c>
       <c r="J176" t="inlineStr">
         <is>
@@ -10323,10 +10323,10 @@
         </is>
       </c>
       <c r="H177" t="n">
-        <v>45.56407282713084</v>
+        <v>45.5465500469921</v>
       </c>
       <c r="I177" t="n">
-        <v>11.50693176186814</v>
+        <v>11.55851844754599</v>
       </c>
       <c r="J177" t="inlineStr">
         <is>
@@ -10379,10 +10379,10 @@
         </is>
       </c>
       <c r="H178" t="n">
-        <v>45.39225128529167</v>
+        <v>45.36490961069684</v>
       </c>
       <c r="I178" t="n">
-        <v>11.83465230668955</v>
+        <v>11.90964730435952</v>
       </c>
       <c r="J178" t="inlineStr">
         <is>
@@ -10435,10 +10435,10 @@
         </is>
       </c>
       <c r="H179" t="n">
-        <v>45.52685973170561</v>
+        <v>45.56645402876486</v>
       </c>
       <c r="I179" t="n">
-        <v>11.5588676199935</v>
+        <v>11.57848712919296</v>
       </c>
       <c r="J179" t="inlineStr">
         <is>
@@ -10491,10 +10491,10 @@
         </is>
       </c>
       <c r="H180" t="n">
-        <v>45.7016128332203</v>
+        <v>45.66376737351595</v>
       </c>
       <c r="I180" t="n">
-        <v>12.23958936968431</v>
+        <v>12.27674901692637</v>
       </c>
       <c r="J180" t="inlineStr">
         <is>
@@ -10547,10 +10547,10 @@
         </is>
       </c>
       <c r="H181" t="n">
-        <v>45.58535468992564</v>
+        <v>45.55298973775317</v>
       </c>
       <c r="I181" t="n">
-        <v>11.54100505473666</v>
+        <v>11.57378565884534</v>
       </c>
       <c r="J181" t="inlineStr">
         <is>
@@ -10603,10 +10603,10 @@
         </is>
       </c>
       <c r="H182" t="n">
-        <v>45.51897315484432</v>
+        <v>45.53036694726358</v>
       </c>
       <c r="I182" t="n">
-        <v>11.56921118210409</v>
+        <v>11.49904740410179</v>
       </c>
       <c r="J182" t="inlineStr">
         <is>
@@ -10659,10 +10659,10 @@
         </is>
       </c>
       <c r="H183" t="n">
-        <v>45.63558373924695</v>
+        <v>45.66955416903522</v>
       </c>
       <c r="I183" t="n">
-        <v>12.22927841883392</v>
+        <v>12.25483965015049</v>
       </c>
       <c r="J183" t="inlineStr">
         <is>
@@ -10767,10 +10767,10 @@
         </is>
       </c>
       <c r="H185" t="n">
-        <v>45.38735426332658</v>
+        <v>45.4234131032881</v>
       </c>
       <c r="I185" t="n">
-        <v>11.8470142185641</v>
+        <v>11.84817683435851</v>
       </c>
       <c r="J185" t="inlineStr">
         <is>
@@ -10823,10 +10823,10 @@
         </is>
       </c>
       <c r="H186" t="n">
-        <v>45.43964555820396</v>
+        <v>45.37360629624386</v>
       </c>
       <c r="I186" t="n">
-        <v>11.84192053830574</v>
+        <v>11.89864768347854</v>
       </c>
       <c r="J186" t="inlineStr">
         <is>
@@ -10879,10 +10879,10 @@
         </is>
       </c>
       <c r="H187" t="n">
-        <v>45.50042480861994</v>
+        <v>45.52173264915437</v>
       </c>
       <c r="I187" t="n">
-        <v>11.5139498588445</v>
+        <v>11.59181393297679</v>
       </c>
       <c r="J187" t="inlineStr">
         <is>
@@ -10935,10 +10935,10 @@
         </is>
       </c>
       <c r="H188" t="n">
-        <v>45.5672839856632</v>
+        <v>45.51127316959194</v>
       </c>
       <c r="I188" t="n">
-        <v>11.5581961546627</v>
+        <v>11.56851511001798</v>
       </c>
       <c r="J188" t="inlineStr">
         <is>
@@ -10991,10 +10991,10 @@
         </is>
       </c>
       <c r="H189" t="n">
-        <v>45.49919144842586</v>
+        <v>45.52605872215928</v>
       </c>
       <c r="I189" t="n">
-        <v>11.54799572471511</v>
+        <v>11.5345338531029</v>
       </c>
       <c r="J189" t="inlineStr">
         <is>
@@ -11047,10 +11047,10 @@
         </is>
       </c>
       <c r="H190" t="n">
-        <v>45.51123650362516</v>
+        <v>45.57065222710738</v>
       </c>
       <c r="I190" t="n">
-        <v>11.56635723748845</v>
+        <v>11.54904663462314</v>
       </c>
       <c r="J190" t="inlineStr">
         <is>
@@ -11103,10 +11103,10 @@
         </is>
       </c>
       <c r="H191" t="n">
-        <v>45.58717520818761</v>
+        <v>45.50100508300459</v>
       </c>
       <c r="I191" t="n">
-        <v>11.50811303800698</v>
+        <v>11.58949717788213</v>
       </c>
       <c r="J191" t="inlineStr">
         <is>
@@ -11159,10 +11159,10 @@
         </is>
       </c>
       <c r="H192" t="n">
-        <v>45.70490125709025</v>
+        <v>45.70328162462787</v>
       </c>
       <c r="I192" t="n">
-        <v>12.23085939505888</v>
+        <v>12.23333732680687</v>
       </c>
       <c r="J192" t="inlineStr">
         <is>
@@ -11215,10 +11215,10 @@
         </is>
       </c>
       <c r="H193" t="n">
-        <v>45.46635195946362</v>
+        <v>45.40363785589561</v>
       </c>
       <c r="I193" t="n">
-        <v>12.29127179539968</v>
+        <v>12.27792353576556</v>
       </c>
       <c r="J193" t="inlineStr">
         <is>
@@ -11271,10 +11271,10 @@
         </is>
       </c>
       <c r="H194" t="n">
-        <v>45.43312011446712</v>
+        <v>45.39587765817384</v>
       </c>
       <c r="I194" t="n">
-        <v>11.88795863463047</v>
+        <v>11.87572983028032</v>
       </c>
       <c r="J194" t="inlineStr">
         <is>
@@ -11327,10 +11327,10 @@
         </is>
       </c>
       <c r="H195" t="n">
-        <v>45.52704703802728</v>
+        <v>45.5530098387316</v>
       </c>
       <c r="I195" t="n">
-        <v>11.58299107182873</v>
+        <v>11.49550840353361</v>
       </c>
       <c r="J195" t="inlineStr">
         <is>
@@ -11383,10 +11383,10 @@
         </is>
       </c>
       <c r="H196" t="n">
-        <v>45.40335937321633</v>
+        <v>45.45133570117293</v>
       </c>
       <c r="I196" t="n">
-        <v>11.86254748955851</v>
+        <v>11.88375824283951</v>
       </c>
       <c r="J196" t="inlineStr">
         <is>
@@ -11439,10 +11439,10 @@
         </is>
       </c>
       <c r="H197" t="n">
-        <v>45.3716636443533</v>
+        <v>45.43783105522845</v>
       </c>
       <c r="I197" t="n">
-        <v>11.83989691689539</v>
+        <v>11.87100959774133</v>
       </c>
       <c r="J197" t="inlineStr">
         <is>
@@ -11495,10 +11495,10 @@
         </is>
       </c>
       <c r="H198" t="n">
-        <v>45.52012288802138</v>
+        <v>45.50122804109356</v>
       </c>
       <c r="I198" t="n">
-        <v>11.52854739897909</v>
+        <v>11.56831753579301</v>
       </c>
       <c r="J198" t="inlineStr"/>
       <c r="K198" t="n">
@@ -11547,10 +11547,10 @@
         </is>
       </c>
       <c r="H199" t="n">
-        <v>45.67496845427814</v>
+        <v>45.65106655200425</v>
       </c>
       <c r="I199" t="n">
-        <v>12.29240779259467</v>
+        <v>12.22684875246339</v>
       </c>
       <c r="J199" t="inlineStr">
         <is>
@@ -11599,10 +11599,10 @@
         </is>
       </c>
       <c r="H200" t="n">
-        <v>45.56438009012513</v>
+        <v>45.54267513510737</v>
       </c>
       <c r="I200" t="n">
-        <v>11.52448024605587</v>
+        <v>11.5852553506783</v>
       </c>
       <c r="J200" t="inlineStr">
         <is>
@@ -11655,10 +11655,10 @@
         </is>
       </c>
       <c r="H201" t="n">
-        <v>45.45132131342087</v>
+        <v>45.41410080771553</v>
       </c>
       <c r="I201" t="n">
-        <v>11.83373894092369</v>
+        <v>11.8769369213795</v>
       </c>
       <c r="J201" t="inlineStr">
         <is>
@@ -11711,10 +11711,10 @@
         </is>
       </c>
       <c r="H202" t="n">
-        <v>45.5811997740626</v>
+        <v>45.58261971669562</v>
       </c>
       <c r="I202" t="n">
-        <v>11.52504604241063</v>
+        <v>11.57808275480635</v>
       </c>
       <c r="J202" t="inlineStr">
         <is>
@@ -11767,10 +11767,10 @@
         </is>
       </c>
       <c r="H203" t="n">
-        <v>45.39856833367515</v>
+        <v>45.44221143490089</v>
       </c>
       <c r="I203" t="n">
-        <v>12.36417543527898</v>
+        <v>12.32942317898853</v>
       </c>
       <c r="J203" t="inlineStr">
         <is>
@@ -11823,10 +11823,10 @@
         </is>
       </c>
       <c r="H204" t="n">
-        <v>45.52257291547325</v>
+        <v>45.5942746296661</v>
       </c>
       <c r="I204" t="n">
-        <v>11.53693183901889</v>
+        <v>11.55596382170885</v>
       </c>
       <c r="J204" t="inlineStr">
         <is>
@@ -11879,10 +11879,10 @@
         </is>
       </c>
       <c r="H205" t="n">
-        <v>45.38289569004106</v>
+        <v>45.43999683713052</v>
       </c>
       <c r="I205" t="n">
-        <v>11.87327319860846</v>
+        <v>11.92313887805316</v>
       </c>
       <c r="J205" t="inlineStr">
         <is>
@@ -11935,10 +11935,10 @@
         </is>
       </c>
       <c r="H206" t="n">
-        <v>45.59021234014</v>
+        <v>45.54756982336438</v>
       </c>
       <c r="I206" t="n">
-        <v>11.56881615470724</v>
+        <v>11.50226262060308</v>
       </c>
       <c r="J206" t="inlineStr">
         <is>
@@ -12043,10 +12043,10 @@
         </is>
       </c>
       <c r="H208" t="n">
-        <v>45.55994833669082</v>
+        <v>45.58918185208231</v>
       </c>
       <c r="I208" t="n">
-        <v>11.5244602729069</v>
+        <v>11.58961428817452</v>
       </c>
       <c r="J208" t="inlineStr">
         <is>
@@ -12099,10 +12099,10 @@
         </is>
       </c>
       <c r="H209" t="n">
-        <v>45.55152507792099</v>
+        <v>45.52174099819236</v>
       </c>
       <c r="I209" t="n">
-        <v>11.59249063054894</v>
+        <v>11.58352656338116</v>
       </c>
       <c r="J209" t="inlineStr">
         <is>
@@ -12155,10 +12155,10 @@
         </is>
       </c>
       <c r="H210" t="n">
-        <v>45.5753016417936</v>
+        <v>45.50156686504408</v>
       </c>
       <c r="I210" t="n">
-        <v>11.58353695372738</v>
+        <v>11.56587534660936</v>
       </c>
       <c r="J210" t="inlineStr">
         <is>
@@ -12211,10 +12211,10 @@
         </is>
       </c>
       <c r="H211" t="n">
-        <v>45.40513437041185</v>
+        <v>45.42127153803388</v>
       </c>
       <c r="I211" t="n">
-        <v>11.8961238131145</v>
+        <v>11.8933659988405</v>
       </c>
       <c r="J211" t="inlineStr">
         <is>
@@ -12267,10 +12267,10 @@
         </is>
       </c>
       <c r="H212" t="n">
-        <v>45.51700270171683</v>
+        <v>45.55794278127709</v>
       </c>
       <c r="I212" t="n">
-        <v>11.514346674783</v>
+        <v>11.52445841974882</v>
       </c>
       <c r="J212" t="inlineStr">
         <is>
@@ -12323,10 +12323,10 @@
         </is>
       </c>
       <c r="H213" t="n">
-        <v>45.36566399905586</v>
+        <v>45.43212763088918</v>
       </c>
       <c r="I213" t="n">
-        <v>11.92080733898641</v>
+        <v>11.83637770218353</v>
       </c>
       <c r="J213" t="inlineStr">
         <is>
@@ -12379,10 +12379,10 @@
         </is>
       </c>
       <c r="H214" t="n">
-        <v>45.55163257215806</v>
+        <v>45.52866760716925</v>
       </c>
       <c r="I214" t="n">
-        <v>11.57138626543324</v>
+        <v>11.58966714643913</v>
       </c>
       <c r="J214" t="inlineStr">
         <is>
@@ -12439,10 +12439,10 @@
         </is>
       </c>
       <c r="H215" t="n">
-        <v>45.51001600482357</v>
+        <v>45.54517503672054</v>
       </c>
       <c r="I215" t="n">
-        <v>11.53286392846858</v>
+        <v>11.50959860871485</v>
       </c>
       <c r="J215" t="inlineStr">
         <is>
@@ -12499,10 +12499,10 @@
         </is>
       </c>
       <c r="H216" t="n">
-        <v>45.50986002510752</v>
+        <v>45.54506057026556</v>
       </c>
       <c r="I216" t="n">
-        <v>11.52449091224969</v>
+        <v>11.50370722601443</v>
       </c>
       <c r="J216" t="inlineStr">
         <is>
@@ -12555,10 +12555,10 @@
         </is>
       </c>
       <c r="H217" t="n">
-        <v>45.42248520100675</v>
+        <v>45.37376783965404</v>
       </c>
       <c r="I217" t="n">
-        <v>11.86792989655506</v>
+        <v>11.90035740511972</v>
       </c>
       <c r="J217" t="inlineStr">
         <is>
@@ -12611,10 +12611,10 @@
         </is>
       </c>
       <c r="H218" t="n">
-        <v>45.54518993183147</v>
+        <v>45.5037179782417</v>
       </c>
       <c r="I218" t="n">
-        <v>11.53661891908458</v>
+        <v>11.50866697989738</v>
       </c>
       <c r="J218" t="inlineStr">
         <is>
@@ -12667,10 +12667,10 @@
         </is>
       </c>
       <c r="H219" t="n">
-        <v>45.57784853259805</v>
+        <v>45.59720826022676</v>
       </c>
       <c r="I219" t="n">
-        <v>11.5623979725327</v>
+        <v>11.54575604138496</v>
       </c>
       <c r="J219" t="inlineStr">
         <is>
@@ -12727,10 +12727,10 @@
         </is>
       </c>
       <c r="H220" t="n">
-        <v>45.50222448500905</v>
+        <v>45.51227770060809</v>
       </c>
       <c r="I220" t="n">
-        <v>11.56970635585868</v>
+        <v>11.58028652623733</v>
       </c>
       <c r="J220" t="inlineStr">
         <is>
@@ -12783,10 +12783,10 @@
         </is>
       </c>
       <c r="H221" t="n">
-        <v>45.57401767437751</v>
+        <v>45.50650340032722</v>
       </c>
       <c r="I221" t="n">
-        <v>11.58262239992792</v>
+        <v>11.51892568336774</v>
       </c>
       <c r="J221" t="inlineStr">
         <is>
@@ -12839,10 +12839,10 @@
         </is>
       </c>
       <c r="H222" t="n">
-        <v>45.52063658563358</v>
+        <v>45.50642746815059</v>
       </c>
       <c r="I222" t="n">
-        <v>11.56025137698109</v>
+        <v>11.51078917019004</v>
       </c>
       <c r="J222" t="inlineStr">
         <is>
@@ -12947,10 +12947,10 @@
         </is>
       </c>
       <c r="H224" t="n">
-        <v>45.57082338152536</v>
+        <v>45.49849505270014</v>
       </c>
       <c r="I224" t="n">
-        <v>11.59277309543397</v>
+        <v>11.54765496637389</v>
       </c>
       <c r="J224" t="inlineStr">
         <is>
@@ -13051,10 +13051,10 @@
         </is>
       </c>
       <c r="H226" t="n">
-        <v>45.593333536717</v>
+        <v>45.58443082928317</v>
       </c>
       <c r="I226" t="n">
-        <v>11.52110219821546</v>
+        <v>11.57826162480449</v>
       </c>
       <c r="J226" t="inlineStr">
         <is>
@@ -13107,10 +13107,10 @@
         </is>
       </c>
       <c r="H227" t="n">
-        <v>45.57047827977479</v>
+        <v>45.52024979885379</v>
       </c>
       <c r="I227" t="n">
-        <v>11.51626693003356</v>
+        <v>11.52587233730721</v>
       </c>
       <c r="J227" t="inlineStr">
         <is>
@@ -13163,10 +13163,10 @@
         </is>
       </c>
       <c r="H228" t="n">
-        <v>45.5703851550674</v>
+        <v>45.57123877511381</v>
       </c>
       <c r="I228" t="n">
-        <v>11.56289279016322</v>
+        <v>11.56628402093287</v>
       </c>
       <c r="J228" t="inlineStr">
         <is>
@@ -13219,10 +13219,10 @@
         </is>
       </c>
       <c r="H229" t="n">
-        <v>45.53045907480365</v>
+        <v>45.55399608530483</v>
       </c>
       <c r="I229" t="n">
-        <v>11.5411548382092</v>
+        <v>11.58003213552871</v>
       </c>
       <c r="J229" t="inlineStr">
         <is>
@@ -13275,10 +13275,10 @@
         </is>
       </c>
       <c r="H230" t="n">
-        <v>45.39335698809052</v>
+        <v>45.43622751249892</v>
       </c>
       <c r="I230" t="n">
-        <v>11.85722185655359</v>
+        <v>11.90666590450052</v>
       </c>
       <c r="J230" t="inlineStr">
         <is>
@@ -13331,10 +13331,10 @@
         </is>
       </c>
       <c r="H231" t="n">
-        <v>45.43290503127141</v>
+        <v>45.48504551063338</v>
       </c>
       <c r="I231" t="n">
-        <v>12.30299655638296</v>
+        <v>12.2659018657852</v>
       </c>
       <c r="J231" t="inlineStr">
         <is>
@@ -13387,10 +13387,10 @@
         </is>
       </c>
       <c r="H232" t="n">
-        <v>45.45119082918661</v>
+        <v>45.36954799528716</v>
       </c>
       <c r="I232" t="n">
-        <v>11.83555634445648</v>
+        <v>11.88684965837305</v>
       </c>
       <c r="J232" t="inlineStr">
         <is>
@@ -13443,10 +13443,10 @@
         </is>
       </c>
       <c r="H233" t="n">
-        <v>45.41839402360176</v>
+        <v>45.42819934669198</v>
       </c>
       <c r="I233" t="n">
-        <v>12.29574337991892</v>
+        <v>12.34712624558524</v>
       </c>
       <c r="J233" t="inlineStr">
         <is>
@@ -13499,10 +13499,10 @@
         </is>
       </c>
       <c r="H234" t="n">
-        <v>45.39977499912978</v>
+        <v>45.36684466703157</v>
       </c>
       <c r="I234" t="n">
-        <v>11.88821464532096</v>
+        <v>11.92051057517748</v>
       </c>
       <c r="J234" t="inlineStr">
         <is>
@@ -13555,10 +13555,10 @@
         </is>
       </c>
       <c r="H235" t="n">
-        <v>45.37411160108667</v>
+        <v>45.3812503283941</v>
       </c>
       <c r="I235" t="n">
-        <v>11.90378002014663</v>
+        <v>11.88910990375812</v>
       </c>
       <c r="J235" t="inlineStr">
         <is>
@@ -13611,10 +13611,10 @@
         </is>
       </c>
       <c r="H236" t="n">
-        <v>45.38728039716194</v>
+        <v>45.44980796652974</v>
       </c>
       <c r="I236" t="n">
-        <v>11.91321600137974</v>
+        <v>11.86487252209042</v>
       </c>
       <c r="J236" t="inlineStr">
         <is>
@@ -13667,10 +13667,10 @@
         </is>
       </c>
       <c r="H237" t="n">
-        <v>45.50579612987006</v>
+        <v>45.50026686298879</v>
       </c>
       <c r="I237" t="n">
-        <v>11.56039787490938</v>
+        <v>11.57365357636955</v>
       </c>
       <c r="J237" t="inlineStr">
         <is>
@@ -13727,10 +13727,10 @@
         </is>
       </c>
       <c r="H238" t="n">
-        <v>45.39998978878562</v>
+        <v>45.42946323328427</v>
       </c>
       <c r="I238" t="n">
-        <v>11.91698839604026</v>
+        <v>11.87531906357259</v>
       </c>
       <c r="J238" t="inlineStr">
         <is>
@@ -13787,10 +13787,10 @@
         </is>
       </c>
       <c r="H239" t="n">
-        <v>45.41480672189458</v>
+        <v>45.35824490549194</v>
       </c>
       <c r="I239" t="n">
-        <v>11.90787061844492</v>
+        <v>11.8953251912311</v>
       </c>
       <c r="J239" t="inlineStr">
         <is>
@@ -13843,10 +13843,10 @@
         </is>
       </c>
       <c r="H240" t="n">
-        <v>45.57763334798659</v>
+        <v>45.57606609215763</v>
       </c>
       <c r="I240" t="n">
-        <v>11.59008155047463</v>
+        <v>11.52315795402445</v>
       </c>
       <c r="J240" t="inlineStr">
         <is>
@@ -13899,10 +13899,10 @@
         </is>
       </c>
       <c r="H241" t="n">
-        <v>45.64179642102379</v>
+        <v>45.66726015144712</v>
       </c>
       <c r="I241" t="n">
-        <v>12.22872280933543</v>
+        <v>12.28316696585205</v>
       </c>
       <c r="J241" t="inlineStr">
         <is>

</xml_diff>